<commit_message>
Record ETM-15493 import retest with transaction date 01-08-2026.
SO-5U4G6031 trx date is 1 Aug 2026 WIB; Benchmark COGS snapshot stays 51.900.

Co-authored-by: Yemima Tifani <Yemimatifani@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/implementation-card/[ETM-15493]/import-expired-manual.xlsx
+++ b/implementation-card/[ETM-15493]/import-expired-manual.xlsx
@@ -43,7 +43,7 @@
     <t>Price</t>
   </si>
   <si>
-    <t>14-08-2026</t>
+    <t>01-08-2026</t>
   </si>
   <si>
     <t>BUYER-OFFLINE-1</t>
@@ -52,7 +52,7 @@
     <t>Store Staging</t>
   </si>
   <si>
-    <t>ETM15493IMP90856980</t>
+    <t>ETM15493IMP92607559</t>
   </si>
   <si>
     <t>STD1001</t>

</xml_diff>